<commit_message>
Atualizacao da selecao de maquina e upload flexivel
</commit_message>
<xml_diff>
--- a/Log_Registro_Anomalias.xlsx
+++ b/Log_Registro_Anomalias.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,71 +413,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Máquina</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Responsável</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>E-mail Destino</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Problema</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>What (Ação)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Why (Por que)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Where (Onde)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>When (Quando)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Who (Quem)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>How (Como)</t>
         </is>
@@ -486,175 +491,195 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>OC-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Krauss Maffei 40/40</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Engenharia de Processos</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>rogerio@grahlconsultoria.com.br</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>falhou</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Pendente Ação Corretiva</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>OC-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>14:37</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Krauss Maffei 40/40</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Pedro Mantovani — Gerente Slitter</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>pedro.mantovani@fastgondolas.com.br</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>falhou</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Pendente Ação Corretiva</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>OC-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>14:37</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Krauss Maffei 40/40</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Rogério Grahl — Engenheiro Consultor</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Rograhl75@gmail.com</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>falhou</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Pendente Ação Corretiva</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>OC-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>14:56</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Krauss Maffei 40/40</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Rogério Grahl — Engenheiro Consultor</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Rograhl75@gmail.com</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t xml:space="preserve">falhou
 </t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Pendente Ação Corretiva</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>